<commit_message>
feat: add power, root and calculator validations
</commit_message>
<xml_diff>
--- a/Plano de Teste - Calculadora.xlsx
+++ b/Plano de Teste - Calculadora.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30203"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B2823A1-B4F4-436B-B551-929449BEE551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF6807C6-9E77-4CDE-9F95-C2CFD5F011D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="150">
   <si>
     <t>TASK 005123 - Implementação da calculadora</t>
   </si>
@@ -156,7 +156,7 @@
     <t>Chamar a função subtrair, e enviar como primeiro parâmetro 2.6, como segundo parâmetro 3.7</t>
   </si>
   <si>
-    <t>A função irá retornar 6.4</t>
+    <t>A função irá retornar -1.1</t>
   </si>
   <si>
     <t>Chamar a função subtrair, e enviar como primeiro parâmetro 'banana', e como segundo parâmetro 12</t>
@@ -279,7 +279,211 @@
     <t>A função irá retornar 4</t>
   </si>
   <si>
-    <t>Data: 27/03/2026</t>
+    <t>Potência</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 2, como segundo parâmetro 3</t>
+  </si>
+  <si>
+    <t>A função irá retornar 8</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 5, como segundo parâmetro 0</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 10, como segundo parâmetro 2</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 3, como segundo parâmetro 4</t>
+  </si>
+  <si>
+    <t>A função irá retornar 81</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro -2, como segundo parâmetro 3</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro -2, como segundo parâmetro 4</t>
+  </si>
+  <si>
+    <t>A função irá retornar 16</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 4, como segundo parâmetro -1</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.25</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 2, como segundo parâmetro -2</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 0, como segundo parâmetro 5</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 1, como segundo parâmetro 50</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 2.5, como segundo parâmetro 2</t>
+  </si>
+  <si>
+    <t>A função irá retornar 6.25</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro -1, como segundo parâmetro 99</t>
+  </si>
+  <si>
+    <t>A função irá retornar -1</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro -1, como segundo parâmetro 100</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 9, como segundo parâmetro 0.5</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 'batata', como segundo parâmetro 2</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 2, como segundo parâmetro 'batata'</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 'banana', como segundo parâmetro 'morango'</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 100, como segundo parâmetro 1</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 7, como segundo parâmetro 3</t>
+  </si>
+  <si>
+    <t>A função irá retornar 343</t>
+  </si>
+  <si>
+    <t>Chamar a função potência, enviar como primeiro parâmetro 12, como segundo parâmetro 2</t>
+  </si>
+  <si>
+    <t>A função irá retornar 144</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 9</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 16</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 25</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 1</t>
+  </si>
+  <si>
+    <t>Raiz</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 0</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 100</t>
+  </si>
+  <si>
+    <t>A função irá retornar 10</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 144</t>
+  </si>
+  <si>
+    <t>A função irá retornar 12</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 0.25</t>
+  </si>
+  <si>
+    <t>A função irá retornar 0.5</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 2.25</t>
+  </si>
+  <si>
+    <t>A função irá retornar 1.5</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro -4</t>
+  </si>
+  <si>
+    <t>A função irá retornar um erro - Não é possível calcular a raiz quadrada de um número negativo</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro -1</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro -100</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 'abacaxi'</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 'melancia'</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 4</t>
+  </si>
+  <si>
+    <t>A função irá retornar 2</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 36</t>
+  </si>
+  <si>
+    <t>A função irá retornar 6</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 49</t>
+  </si>
+  <si>
+    <t>A função irá retornar 7</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 64</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 81</t>
+  </si>
+  <si>
+    <t>A função irá retornar 9</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 121</t>
+  </si>
+  <si>
+    <t>A função irá retornar 11</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 169</t>
+  </si>
+  <si>
+    <t>A função irá retornar 13</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 400</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 625</t>
+  </si>
+  <si>
+    <t>A função irá retornar 25</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 900</t>
+  </si>
+  <si>
+    <t>A função irá retornar 30</t>
+  </si>
+  <si>
+    <t>Chamar a função raiz, enviar como parâmetro 10000</t>
+  </si>
+  <si>
+    <t>Data: 15/06/2026</t>
   </si>
   <si>
     <t>Autor: Natalia S. Rodrigues</t>
@@ -289,7 +493,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,12 +539,6 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -409,7 +607,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -446,24 +644,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <top style="thin">
         <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
+      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -474,8 +661,41 @@
         <color rgb="FF000000"/>
       </left>
       <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -499,10 +719,10 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -512,9 +732,8 @@
     <xf numFmtId="4" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -523,17 +742,11 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -544,12 +757,25 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -887,7 +1113,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -899,47 +1125,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
-      <c r="A1" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
     </row>
     <row r="4" spans="1:6" ht="57.75" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
     </row>
     <row r="5" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -958,11 +1184,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="36" customHeight="1">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:6" ht="39" customHeight="1">
+      <c r="A6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="3">
@@ -978,9 +1204,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="36" customHeight="1">
-      <c r="A7" s="25"/>
-      <c r="B7" s="18"/>
+    <row r="7" spans="1:6" ht="39" customHeight="1">
+      <c r="A7" s="20"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="3">
         <v>2</v>
       </c>
@@ -994,9 +1220,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="36" customHeight="1">
-      <c r="A8" s="25"/>
-      <c r="B8" s="18"/>
+    <row r="8" spans="1:6" ht="39" customHeight="1">
+      <c r="A8" s="20"/>
+      <c r="B8" s="23"/>
       <c r="C8" s="3">
         <v>3</v>
       </c>
@@ -1010,9 +1236,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="36" customHeight="1">
-      <c r="A9" s="25"/>
-      <c r="B9" s="18"/>
+    <row r="9" spans="1:6" ht="39" customHeight="1">
+      <c r="A9" s="20"/>
+      <c r="B9" s="23"/>
       <c r="C9" s="3">
         <v>4</v>
       </c>
@@ -1026,9 +1252,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="36" customHeight="1">
-      <c r="A10" s="25"/>
-      <c r="B10" s="18"/>
+    <row r="10" spans="1:6" ht="39" customHeight="1">
+      <c r="A10" s="20"/>
+      <c r="B10" s="23"/>
       <c r="C10" s="3">
         <v>5</v>
       </c>
@@ -1042,9 +1268,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="36" customHeight="1">
-      <c r="A11" s="25"/>
-      <c r="B11" s="18"/>
+    <row r="11" spans="1:6" ht="39" customHeight="1">
+      <c r="A11" s="20"/>
+      <c r="B11" s="23"/>
       <c r="C11" s="3">
         <v>6</v>
       </c>
@@ -1058,9 +1284,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="36" customHeight="1">
-      <c r="A12" s="25"/>
-      <c r="B12" s="18"/>
+    <row r="12" spans="1:6" ht="39" customHeight="1">
+      <c r="A12" s="20"/>
+      <c r="B12" s="23"/>
       <c r="C12" s="3">
         <v>7</v>
       </c>
@@ -1074,9 +1300,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="36" customHeight="1">
-      <c r="A13" s="25"/>
-      <c r="B13" s="18"/>
+    <row r="13" spans="1:6" ht="39" customHeight="1">
+      <c r="A13" s="20"/>
+      <c r="B13" s="23"/>
       <c r="C13" s="3">
         <v>8</v>
       </c>
@@ -1090,9 +1316,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="36" customHeight="1">
-      <c r="A14" s="25"/>
-      <c r="B14" s="18"/>
+    <row r="14" spans="1:6" ht="39" customHeight="1">
+      <c r="A14" s="20"/>
+      <c r="B14" s="23"/>
       <c r="C14" s="3">
         <v>9</v>
       </c>
@@ -1106,9 +1332,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="36" customHeight="1">
-      <c r="A15" s="25"/>
-      <c r="B15" s="19"/>
+    <row r="15" spans="1:6" ht="39" customHeight="1">
+      <c r="A15" s="20"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="3">
         <v>10</v>
       </c>
@@ -1122,9 +1348,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="36" customHeight="1">
-      <c r="A16" s="25"/>
-      <c r="B16" s="17" t="s">
+    <row r="16" spans="1:6" ht="39" customHeight="1">
+      <c r="A16" s="20"/>
+      <c r="B16" s="22" t="s">
         <v>30</v>
       </c>
       <c r="C16" s="3">
@@ -1140,9 +1366,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="36" customHeight="1">
-      <c r="A17" s="25"/>
-      <c r="B17" s="18"/>
+    <row r="17" spans="1:6" ht="39" customHeight="1">
+      <c r="A17" s="20"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="3">
         <v>12</v>
       </c>
@@ -1156,9 +1382,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="36" customHeight="1">
-      <c r="A18" s="25"/>
-      <c r="B18" s="18"/>
+    <row r="18" spans="1:6" ht="39" customHeight="1">
+      <c r="A18" s="20"/>
+      <c r="B18" s="23"/>
       <c r="C18" s="3">
         <v>13</v>
       </c>
@@ -1172,9 +1398,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="36" customHeight="1">
-      <c r="A19" s="25"/>
-      <c r="B19" s="18"/>
+    <row r="19" spans="1:6" ht="39" customHeight="1">
+      <c r="A19" s="20"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="3">
         <v>14</v>
       </c>
@@ -1188,9 +1414,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="36" customHeight="1">
-      <c r="A20" s="25"/>
-      <c r="B20" s="18"/>
+    <row r="20" spans="1:6" ht="39" customHeight="1">
+      <c r="A20" s="20"/>
+      <c r="B20" s="23"/>
       <c r="C20" s="3">
         <v>15</v>
       </c>
@@ -1204,9 +1430,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="36" customHeight="1">
-      <c r="A21" s="25"/>
-      <c r="B21" s="18"/>
+    <row r="21" spans="1:6" ht="39" customHeight="1">
+      <c r="A21" s="20"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="3">
         <v>16</v>
       </c>
@@ -1220,9 +1446,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="36" customHeight="1">
-      <c r="A22" s="25"/>
-      <c r="B22" s="18"/>
+    <row r="22" spans="1:6" ht="39" customHeight="1">
+      <c r="A22" s="20"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="3">
         <v>17</v>
       </c>
@@ -1236,9 +1462,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="36" customHeight="1">
-      <c r="A23" s="25"/>
-      <c r="B23" s="18"/>
+    <row r="23" spans="1:6" ht="39" customHeight="1">
+      <c r="A23" s="20"/>
+      <c r="B23" s="23"/>
       <c r="C23" s="3">
         <v>18</v>
       </c>
@@ -1252,9 +1478,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="36" customHeight="1">
-      <c r="A24" s="25"/>
-      <c r="B24" s="18"/>
+    <row r="24" spans="1:6" ht="39" customHeight="1">
+      <c r="A24" s="20"/>
+      <c r="B24" s="23"/>
       <c r="C24" s="3">
         <v>19</v>
       </c>
@@ -1268,9 +1494,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="36" customHeight="1">
-      <c r="A25" s="25"/>
-      <c r="B25" s="19"/>
+    <row r="25" spans="1:6" ht="39" customHeight="1">
+      <c r="A25" s="20"/>
+      <c r="B25" s="24"/>
       <c r="C25" s="3">
         <v>20</v>
       </c>
@@ -1284,9 +1510,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="36" customHeight="1">
-      <c r="A26" s="25"/>
-      <c r="B26" s="17" t="s">
+    <row r="26" spans="1:6" ht="39" customHeight="1">
+      <c r="A26" s="20"/>
+      <c r="B26" s="22" t="s">
         <v>47</v>
       </c>
       <c r="C26" s="3">
@@ -1302,9 +1528,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="36" customHeight="1">
-      <c r="A27" s="25"/>
-      <c r="B27" s="18"/>
+    <row r="27" spans="1:6" ht="39" customHeight="1">
+      <c r="A27" s="20"/>
+      <c r="B27" s="23"/>
       <c r="C27" s="3">
         <v>22</v>
       </c>
@@ -1318,9 +1544,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="36" customHeight="1">
-      <c r="A28" s="25"/>
-      <c r="B28" s="18"/>
+    <row r="28" spans="1:6" ht="39" customHeight="1">
+      <c r="A28" s="20"/>
+      <c r="B28" s="23"/>
       <c r="C28" s="3">
         <v>23</v>
       </c>
@@ -1334,9 +1560,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="36" customHeight="1">
-      <c r="A29" s="25"/>
-      <c r="B29" s="18"/>
+    <row r="29" spans="1:6" ht="39" customHeight="1">
+      <c r="A29" s="20"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="3">
         <v>24</v>
       </c>
@@ -1350,9 +1576,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="36" customHeight="1">
-      <c r="A30" s="25"/>
-      <c r="B30" s="18"/>
+    <row r="30" spans="1:6" ht="39" customHeight="1">
+      <c r="A30" s="20"/>
+      <c r="B30" s="23"/>
       <c r="C30" s="3">
         <v>25</v>
       </c>
@@ -1366,9 +1592,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="36" customHeight="1">
-      <c r="A31" s="25"/>
-      <c r="B31" s="18"/>
+    <row r="31" spans="1:6" ht="39" customHeight="1">
+      <c r="A31" s="20"/>
+      <c r="B31" s="23"/>
       <c r="C31" s="3">
         <v>26</v>
       </c>
@@ -1382,9 +1608,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="36" customHeight="1">
-      <c r="A32" s="25"/>
-      <c r="B32" s="18"/>
+    <row r="32" spans="1:6" ht="39" customHeight="1">
+      <c r="A32" s="20"/>
+      <c r="B32" s="23"/>
       <c r="C32" s="3">
         <v>27</v>
       </c>
@@ -1398,9 +1624,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="36" customHeight="1">
-      <c r="A33" s="25"/>
-      <c r="B33" s="18"/>
+    <row r="33" spans="1:6" ht="39" customHeight="1">
+      <c r="A33" s="20"/>
+      <c r="B33" s="23"/>
       <c r="C33" s="3">
         <v>28</v>
       </c>
@@ -1414,9 +1640,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="36" customHeight="1">
-      <c r="A34" s="25"/>
-      <c r="B34" s="18"/>
+    <row r="34" spans="1:6" ht="39" customHeight="1">
+      <c r="A34" s="20"/>
+      <c r="B34" s="23"/>
       <c r="C34" s="3">
         <v>29</v>
       </c>
@@ -1430,25 +1656,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="36" customHeight="1">
-      <c r="A35" s="25"/>
-      <c r="B35" s="18"/>
+    <row r="35" spans="1:6" ht="39" customHeight="1">
+      <c r="A35" s="20"/>
+      <c r="B35" s="23"/>
       <c r="C35" s="3">
         <v>30</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="D35" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="E35" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F35" s="15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="36" customHeight="1">
-      <c r="A36" s="26"/>
-      <c r="B36" s="17" t="s">
+      <c r="F35" s="14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="39" customHeight="1">
+      <c r="A36" s="20"/>
+      <c r="B36" s="22" t="s">
         <v>64</v>
       </c>
       <c r="C36" s="3">
@@ -1464,9 +1690,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="36" customHeight="1">
-      <c r="A37" s="26"/>
-      <c r="B37" s="18"/>
+    <row r="37" spans="1:6" ht="39" customHeight="1">
+      <c r="A37" s="20"/>
+      <c r="B37" s="23"/>
       <c r="C37" s="3">
         <v>32</v>
       </c>
@@ -1480,13 +1706,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="36" customHeight="1">
-      <c r="A38" s="26"/>
-      <c r="B38" s="18"/>
+    <row r="38" spans="1:6" ht="39" customHeight="1">
+      <c r="A38" s="20"/>
+      <c r="B38" s="23"/>
       <c r="C38" s="3">
         <v>33</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="12" t="s">
         <v>68</v>
       </c>
       <c r="E38" s="4" t="s">
@@ -1496,9 +1722,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="36" customHeight="1">
-      <c r="A39" s="26"/>
-      <c r="B39" s="18"/>
+    <row r="39" spans="1:6" ht="39" customHeight="1">
+      <c r="A39" s="20"/>
+      <c r="B39" s="23"/>
       <c r="C39" s="3">
         <v>34</v>
       </c>
@@ -1512,9 +1738,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="36" customHeight="1">
-      <c r="A40" s="26"/>
-      <c r="B40" s="18"/>
+    <row r="40" spans="1:6" ht="39" customHeight="1">
+      <c r="A40" s="20"/>
+      <c r="B40" s="23"/>
       <c r="C40" s="3">
         <v>35</v>
       </c>
@@ -1528,9 +1754,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="36" customHeight="1">
-      <c r="A41" s="26"/>
-      <c r="B41" s="18"/>
+    <row r="41" spans="1:6" ht="39" customHeight="1">
+      <c r="A41" s="20"/>
+      <c r="B41" s="23"/>
       <c r="C41" s="3">
         <v>36</v>
       </c>
@@ -1544,9 +1770,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="36" customHeight="1">
-      <c r="A42" s="26"/>
-      <c r="B42" s="18"/>
+    <row r="42" spans="1:6" ht="39" customHeight="1">
+      <c r="A42" s="20"/>
+      <c r="B42" s="23"/>
       <c r="C42" s="3">
         <v>37</v>
       </c>
@@ -1560,9 +1786,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="36" customHeight="1">
-      <c r="A43" s="26"/>
-      <c r="B43" s="18"/>
+    <row r="43" spans="1:6" ht="39" customHeight="1">
+      <c r="A43" s="20"/>
+      <c r="B43" s="23"/>
       <c r="C43" s="3">
         <v>38</v>
       </c>
@@ -1576,29 +1802,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="36" customHeight="1">
-      <c r="A44" s="26"/>
-      <c r="B44" s="18"/>
+    <row r="44" spans="1:6" ht="39" customHeight="1">
+      <c r="A44" s="20"/>
+      <c r="B44" s="23"/>
       <c r="C44" s="3">
         <v>39</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="E44" s="13" t="s">
         <v>77</v>
       </c>
       <c r="F44" s="5" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="36" customHeight="1">
-      <c r="A45" s="12"/>
-      <c r="B45" s="19"/>
+    <row r="45" spans="1:6" ht="39" customHeight="1">
+      <c r="A45" s="20"/>
+      <c r="B45" s="23"/>
       <c r="C45" s="3">
         <v>40</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="D45" s="15" t="s">
         <v>78</v>
       </c>
       <c r="E45" s="4" t="s">
@@ -1608,37 +1834,763 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="13.5" customHeight="1">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="10"/>
-    </row>
-    <row r="47" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A47" s="11" t="s">
+    <row r="46" spans="1:6" ht="39" customHeight="1">
+      <c r="A46" s="20"/>
+      <c r="B46" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="16" t="s">
+      <c r="C46" s="3">
+        <v>41</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D47" s="16"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
+      <c r="E46" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F46" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="39" customHeight="1">
+      <c r="A47" s="20"/>
+      <c r="B47" s="25"/>
+      <c r="C47" s="3">
+        <v>42</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F47" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="39" customHeight="1">
+      <c r="A48" s="20"/>
+      <c r="B48" s="25"/>
+      <c r="C48" s="3">
+        <v>43</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="39" customHeight="1">
+      <c r="A49" s="20"/>
+      <c r="B49" s="25"/>
+      <c r="C49" s="3">
+        <v>44</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F49" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="39" customHeight="1">
+      <c r="A50" s="20"/>
+      <c r="B50" s="25"/>
+      <c r="C50" s="3">
+        <v>45</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F50" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="39" customHeight="1">
+      <c r="A51" s="20"/>
+      <c r="B51" s="25"/>
+      <c r="C51" s="3">
+        <v>46</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F51" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="39" customHeight="1">
+      <c r="A52" s="20"/>
+      <c r="B52" s="25"/>
+      <c r="C52" s="3">
+        <v>47</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F52" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="39" customHeight="1">
+      <c r="A53" s="20"/>
+      <c r="B53" s="25"/>
+      <c r="C53" s="3">
+        <v>48</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F53" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="39" customHeight="1">
+      <c r="A54" s="20"/>
+      <c r="B54" s="25"/>
+      <c r="C54" s="3">
+        <v>49</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F54" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="39" customHeight="1">
+      <c r="A55" s="20"/>
+      <c r="B55" s="25"/>
+      <c r="C55" s="3">
+        <v>50</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F55" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="39" customHeight="1">
+      <c r="A56" s="20"/>
+      <c r="B56" s="25"/>
+      <c r="C56" s="3">
+        <v>51</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F56" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="39" customHeight="1">
+      <c r="A57" s="20"/>
+      <c r="B57" s="25"/>
+      <c r="C57" s="3">
+        <v>52</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F57" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="39" customHeight="1">
+      <c r="A58" s="20"/>
+      <c r="B58" s="25"/>
+      <c r="C58" s="3">
+        <v>53</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F58" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="39" customHeight="1">
+      <c r="A59" s="20"/>
+      <c r="B59" s="25"/>
+      <c r="C59" s="3">
+        <v>54</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F59" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="39" customHeight="1">
+      <c r="A60" s="20"/>
+      <c r="B60" s="25"/>
+      <c r="C60" s="3">
+        <v>55</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F60" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="39" customHeight="1">
+      <c r="A61" s="20"/>
+      <c r="B61" s="25"/>
+      <c r="C61" s="3">
+        <v>56</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F61" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="39" customHeight="1">
+      <c r="A62" s="20"/>
+      <c r="B62" s="25"/>
+      <c r="C62" s="3">
+        <v>57</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F62" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="39" customHeight="1">
+      <c r="A63" s="20"/>
+      <c r="B63" s="25"/>
+      <c r="C63" s="3">
+        <v>58</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="39" customHeight="1">
+      <c r="A64" s="20"/>
+      <c r="B64" s="25"/>
+      <c r="C64" s="3">
+        <v>59</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F64" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="39" customHeight="1">
+      <c r="A65" s="20"/>
+      <c r="B65" s="25"/>
+      <c r="C65" s="3">
+        <v>60</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F65" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="39" customHeight="1">
+      <c r="A66" s="20"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="3">
+        <v>61</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F66" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="39" customHeight="1">
+      <c r="A67" s="20"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="3">
+        <v>62</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F67" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="39" customHeight="1">
+      <c r="A68" s="20"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="3">
+        <v>63</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F68" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="39" customHeight="1">
+      <c r="A69" s="20"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="3">
+        <v>64</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F69" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="39" customHeight="1">
+      <c r="A70" s="20"/>
+      <c r="B70" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="C70" s="3">
+        <v>65</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F70" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="39" customHeight="1">
+      <c r="A71" s="20"/>
+      <c r="B71" s="23"/>
+      <c r="C71" s="3">
+        <v>66</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="F71" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="39" customHeight="1">
+      <c r="A72" s="20"/>
+      <c r="B72" s="23"/>
+      <c r="C72" s="3">
+        <v>67</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F72" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="39" customHeight="1">
+      <c r="A73" s="20"/>
+      <c r="B73" s="23"/>
+      <c r="C73" s="3">
+        <v>68</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F73" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="39" customHeight="1">
+      <c r="A74" s="20"/>
+      <c r="B74" s="23"/>
+      <c r="C74" s="3">
+        <v>69</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F74" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="55.5" customHeight="1">
+      <c r="A75" s="20"/>
+      <c r="B75" s="23"/>
+      <c r="C75" s="3">
+        <v>70</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F75" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="54" customHeight="1">
+      <c r="A76" s="20"/>
+      <c r="B76" s="23"/>
+      <c r="C76" s="3">
+        <v>71</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F76" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="54.75" customHeight="1">
+      <c r="A77" s="20"/>
+      <c r="B77" s="23"/>
+      <c r="C77" s="3">
+        <v>72</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F77" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="39" customHeight="1">
+      <c r="A78" s="20"/>
+      <c r="B78" s="23"/>
+      <c r="C78" s="3">
+        <v>73</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F78" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="39" customHeight="1">
+      <c r="A79" s="20"/>
+      <c r="B79" s="23"/>
+      <c r="C79" s="3">
+        <v>74</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F79" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="39" customHeight="1">
+      <c r="A80" s="20"/>
+      <c r="B80" s="23"/>
+      <c r="C80" s="3">
+        <v>75</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F80" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="39" customHeight="1">
+      <c r="A81" s="20"/>
+      <c r="B81" s="23"/>
+      <c r="C81" s="3">
+        <v>76</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F81" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="39" customHeight="1">
+      <c r="A82" s="20"/>
+      <c r="B82" s="23"/>
+      <c r="C82" s="3">
+        <v>77</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F82" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="39" customHeight="1">
+      <c r="A83" s="20"/>
+      <c r="B83" s="23"/>
+      <c r="C83" s="3">
+        <v>78</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F83" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="39" customHeight="1">
+      <c r="A84" s="20"/>
+      <c r="B84" s="23"/>
+      <c r="C84" s="3">
+        <v>79</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F84" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="39" customHeight="1">
+      <c r="A85" s="20"/>
+      <c r="B85" s="23"/>
+      <c r="C85" s="3">
+        <v>80</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F85" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="39" customHeight="1">
+      <c r="A86" s="20"/>
+      <c r="B86" s="23"/>
+      <c r="C86" s="3">
+        <v>81</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E86" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F86" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="39" customHeight="1">
+      <c r="A87" s="20"/>
+      <c r="B87" s="23"/>
+      <c r="C87" s="3">
+        <v>82</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F87" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="39" customHeight="1">
+      <c r="A88" s="20"/>
+      <c r="B88" s="23"/>
+      <c r="C88" s="3">
+        <v>83</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F88" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="39" customHeight="1">
+      <c r="A89" s="20"/>
+      <c r="B89" s="23"/>
+      <c r="C89" s="3">
+        <v>84</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="F89" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="39" customHeight="1">
+      <c r="A90" s="20"/>
+      <c r="B90" s="24"/>
+      <c r="C90" s="3">
+        <v>85</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F90" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="13.5" customHeight="1">
+      <c r="A91" s="7"/>
+      <c r="B91" s="7"/>
+      <c r="C91" s="8"/>
+      <c r="D91" s="9"/>
+      <c r="E91" s="10"/>
+    </row>
+    <row r="92" spans="1:6" ht="17.25" customHeight="1">
+      <c r="A92" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B92" s="11"/>
+      <c r="C92" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="D92" s="21"/>
+      <c r="E92" s="11"/>
+      <c r="F92" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
+    <mergeCell ref="C92:D92"/>
+    <mergeCell ref="B6:B15"/>
+    <mergeCell ref="B16:B25"/>
+    <mergeCell ref="B26:B35"/>
+    <mergeCell ref="B36:B45"/>
+    <mergeCell ref="B46:B65"/>
+    <mergeCell ref="B70:B90"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A6:A44"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="B6:B15"/>
-    <mergeCell ref="B16:B25"/>
-    <mergeCell ref="B26:B35"/>
-    <mergeCell ref="B36:B45"/>
+    <mergeCell ref="A6:A90"/>
   </mergeCells>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>